<commit_message>
feat: add focus recipes ranking and cooking progression tracking
- Rank unlocked and locked cooking recipes by ungifted recipient impact
- Add recipe sources database with unlock locations and requirements
- Separate owned vs craftable allocation passes in max-relationship strategy
- Prioritize multi-NPC coverage in slot minimization regardless of status
- Export focus recipes in terminal summaries and dedicated Excel worksheet
- Add comprehensive test suites with 425 tests and update gitignore
</commit_message>
<xml_diff>
--- a/exports/daily_gift_bag_plan.xlsx
+++ b/exports/daily_gift_bag_plan.xlsx
@@ -11,12 +11,14 @@
     <sheet name="NPC Gift Progress" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="All Remaining Items" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Gift Completion Matrix" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Focus Recipes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Bag Plan'!$A$1:$O$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Bag Plan'!$A$1:$O$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NPC Gift Progress'!$A$1:$M$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Remaining Items'!$A$1:$L$238</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Gift Completion Matrix'!$A$1:$AK$439</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Focus Recipes'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -549,20 +551,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
     <col width="41" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
@@ -651,58 +653,58 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Golden Sheep Wool</t>
+          <t>Golden Cheesecake</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>golden_sheep_wool</t>
+          <t>golden_cheesecake</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Golden Butter [← 8× Golden Milk]</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Louis, Merri, Wheedle</t>
+          <t>Darcy, Taliferro, Wheedle</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Louis, Merri</t>
+          <t>Darcy, Landen, Ryis</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Wheedle</t>
+          <t>Balor, Caldarus, Taliferro, Wheedle</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Louis, Merri</t>
+          <t>Darcy, Landen, Ryis</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Wheedle</t>
+          <t>Balor, Caldarus, Taliferro, Wheedle</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr"/>
       <c r="M2" s="4" t="inlineStr"/>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>animal_fibre, animal_harvest, animal_product, ranching, wool</t>
+          <t>baked_dessert, food</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr"/>
@@ -712,50 +714,58 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Crystal Berry Pie</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>crystal_berry_pie</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Crystal Berry Pie [← 3× Crystal Berries, 3× Flour, 3× Chicken Egg, 3× Sugar]</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Darcy</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
+          <t>Stillwell</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Stillwell</t>
+        </is>
+      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Darcy, Henrietta</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr"/>
+          <t>Elsie, Reina</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Stillwell</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Darcy, Henrietta</t>
+          <t>Elsie, Reina</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="4" t="inlineStr"/>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>citrus, crop</t>
+          <t>baked_dessert, food</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr"/>
@@ -774,12 +784,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Glowberry Cookies</t>
+          <t>Golden Sheep Wool</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>glowberry_cookies</t>
+          <t>golden_sheep_wool</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -789,26 +799,30 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Taliferro</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Dell, Taliferro</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr"/>
+          <t>Louis, Merri</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Louis, Merri</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Louis, Merri</t>
+        </is>
+      </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Dell, Taliferro</t>
+          <t>Wheedle</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>baked_dessert, food</t>
+          <t>animal_fibre, animal_harvest, animal_product, ranching, wool</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr"/>
@@ -818,54 +832,58 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Golden Horse Hair</t>
+          <t>Jam Sandwich</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>golden_horse_hair</t>
+          <t>jam_sandwich</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
+          <t>Wild Berry Jam [← 18× Wild Berries, 3× Sugar]</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Landen, Ryis</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr"/>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Josephine, Luc</t>
+        </is>
+      </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Landen, Ryis</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Wheedle</t>
+          <t>Josephine, Luc</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr"/>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>animal_fibre, animal_harvest, animal_product, ranching</t>
+          <t>food, hand_crafted_dish</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr"/>
@@ -875,50 +893,58 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Fire Crystal</t>
+          <t>Crispy Fried Earthshroom</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>fire_crystal</t>
+          <t>crispy_fried_earthshroom</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Crispy Fried Earthshroom [← 2× Earthshroom, 2× Flour, 2× Oil]</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Stillwell</t>
+          <t>Vera</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Stillwell</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr"/>
+          <t>Hemlock</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Vera</t>
+        </is>
+      </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Stillwell</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr"/>
+          <t>Hemlock</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Vera</t>
+        </is>
+      </c>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr"/>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>archaeology</t>
+          <t>food, mushroomy, snack</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr"/>
@@ -928,26 +954,26 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Fennel</t>
+          <t>Miner's Mushroom Stew</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>fennel</t>
+          <t>miners_mushroom_stew</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Miner's Mushroom Stew [← 2× Upper Mines Mushroom, 2× Cave Mushroom]</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -958,20 +984,20 @@
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Zorel</t>
+          <t>Olric, Zorel</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Zorel</t>
+          <t>Olric, Zorel</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="4" t="inlineStr"/>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>forageable</t>
+          <t>food, mushroomy, stew</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr"/>
@@ -981,50 +1007,58 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Simmered Daikon</t>
+          <t>Grilled Corn</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>simmered_daikon</t>
+          <t>grilled_corn</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
+          <t>Grilled Corn [← 2× Corn]</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Vera</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Henrietta</t>
+        </is>
+      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Vera</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr"/>
+          <t>Nora</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Henrietta</t>
+        </is>
+      </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Vera</t>
+          <t>Nora</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr"/>
       <c r="M8" s="4" t="inlineStr"/>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>food, simmered_dish</t>
+          <t>food, greens</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr"/>
@@ -1034,50 +1068,58 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Breaded Catfish</t>
+          <t>Deep Sea Soup</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>breaded_catfish</t>
+          <t>deep_sea_soup</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
+          <t>Deep Sea Soup [← 1× Jade Dulse, 1× Mines Mussels, 1× Underseaweed]</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Reina</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr"/>
+          <t>Valen</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Terithia</t>
+        </is>
+      </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Reina</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr"/>
+          <t>Valen</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Landen, Reina, Terithia</t>
+        </is>
+      </c>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="4" t="inlineStr"/>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>fishy, food, fried_dish, no_inn_plate</t>
+          <t>food, soup</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr"/>
@@ -1091,50 +1133,46 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Incredibly Hot Pot</t>
+          <t>Dog Treat</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>incredibly_hot_pot</t>
+          <t>dog_treat</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
+          <t>Dog Treat [← 1× Trout]</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Hemlock</t>
+          <t>Dozy</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr"/>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Hemlock, Josephine</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Caldarus, Taliferro</t>
-        </is>
-      </c>
+          <t>Dozy</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr"/>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="4" t="inlineStr"/>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>food, mushroomy, simmered_dish</t>
+          <t>animal_feed, cat_treat, milled_animal_feed, milling, weird_gift</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr"/>
@@ -1148,38 +1186,38 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Perfect Silver Ore</t>
+          <t>Clam Chowder</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>perfect_silver_ore</t>
+          <t>clam_chowder</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
+          <t>Butter [← 2× Milk]</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Olric</t>
+          <t>Errol</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr"/>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Olric</t>
+          <t>Errol</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr"/>
@@ -1187,7 +1225,7 @@
       <c r="M11" s="4" t="inlineStr"/>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>archaeology, material, ore</t>
+          <t>drink_sound, fishy, food, soup</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr"/>
@@ -1201,50 +1239,46 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Spell Fruit Parfait</t>
+          <t>Golden Mayonnaise</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>spell_fruit_parfait</t>
+          <t>golden_mayonnaise</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
+          <t>Golden Mayonnaise [← 2× Golden Egg]</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Juniper</t>
+          <t>Hayden</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr"/>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Juniper, Seridia, Stillwell, Taliferro</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>Caldarus</t>
-        </is>
-      </c>
+          <t>Hayden</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="4" t="inlineStr"/>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>food, frozen_dessert</t>
+          <t>animal_product, golden_mayonnaise, milling, ranching</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr"/>
@@ -1263,12 +1297,12 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Cod</t>
+          <t>Spell Fruit Parfait</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>cod</t>
+          <t>spell_fruit_parfait</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1281,23 +1315,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Dozy</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Juniper</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Juniper, Seridia, Stillwell, Taliferro</t>
+        </is>
+      </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Dozy</t>
+          <t>Caldarus</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="4" t="inlineStr"/>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>fishable, fishy</t>
+          <t>food, frozen_dessert</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr"/>
@@ -1364,22 +1402,22 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Rose Tea</t>
+          <t>Pudding</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>rose_tea</t>
+          <t>pudding</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pudding [← 2× Chicken Egg, 1× Sugar, 1× Milk]</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1390,20 +1428,20 @@
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Celine</t>
+          <t>Maple</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr"/>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Celine</t>
+          <t>Dell, Maple</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="4" t="inlineStr"/>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>caffeine, drink, drink_sound, food, hot_drink</t>
+          <t>candy, food</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr"/>
@@ -1417,22 +1455,22 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Soy Sauce</t>
+          <t>Lemonade</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>soy_sauce</t>
+          <t>lemonade</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Lemonade [← 1× Lemon, 1× Sugar]</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1443,20 +1481,20 @@
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Josephine</t>
+          <t>Adeline</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr"/>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Josephine</t>
+          <t>Adeline</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>material, pantry</t>
+          <t>citrus, cold_drink, drink, drink_sound, food, no_inn_plate</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr"/>
@@ -1475,12 +1513,12 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Sweetroot</t>
+          <t>Rose Tea</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>sweetroot</t>
+          <t>rose_tea</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1496,20 +1534,20 @@
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Valen</t>
+          <t>Celine</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Valen</t>
+          <t>Celine</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="4" t="inlineStr"/>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>forageable, mines_forageable</t>
+          <t>caffeine, drink, drink_sound, food, hot_drink</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr"/>
@@ -1528,12 +1566,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Frost Lily</t>
+          <t>Iron Ingot</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>frost_lily</t>
+          <t>iron_ingot</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1549,20 +1587,20 @@
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Balor</t>
+          <t>March</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr"/>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Balor, Louis</t>
+          <t>March</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>flower, forageable</t>
+          <t>blacksmithing, ingot</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr"/>
@@ -1576,22 +1614,22 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Iron Ingot</t>
+          <t>Monster Cookies</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>iron_ingot</t>
+          <t>monster_cookie</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Monster Cookie [← 1× Monster Powder, 1× Monster Core, 1× Sugar]</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1602,20 +1640,20 @@
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>March</t>
+          <t>Seridia</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr"/>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>March</t>
+          <t>Seridia, Stillwell</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr"/>
       <c r="M19" s="4" t="inlineStr"/>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>blacksmithing, ingot</t>
+          <t>baked_dessert, food</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr"/>
@@ -1629,22 +1667,22 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>HAVE</t>
+          <t>CRAFT</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Pond Skater</t>
+          <t>Peaches and Cream</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>pond_skater</t>
+          <t>peaches_and_cream</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Peaches and Cream [← 1× Peach, 1× Sugar, 1× Milk]</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1655,352 +1693,26 @@
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Luc</t>
+          <t>Eiland</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr"/>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Luc</t>
+          <t>Eiland</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>bugs</t>
+          <t>food, hand_crafted_dessert</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr"/>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>HAVE</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Cherry Tart</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>cherry_tart</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Elsie</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr"/>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>Elsie</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr"/>
-      <c r="M21" s="4" t="inlineStr"/>
-      <c r="N21" s="3" t="inlineStr">
-        <is>
-          <t>baked_dessert, food</t>
-        </is>
-      </c>
-      <c r="O21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>HAVE</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Deep Sea Soup</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>deep_sea_soup</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>Terithia</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>Valen</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>Landen, Reina, Terithia</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr"/>
-      <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" s="3" t="inlineStr">
-        <is>
-          <t>food, soup</t>
-        </is>
-      </c>
-      <c r="O22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>HAVE</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Purple Mushroom</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>purple_mushroom</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>Seridia</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>Seridia</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr"/>
-      <c r="M23" s="4" t="inlineStr"/>
-      <c r="N23" s="3" t="inlineStr">
-        <is>
-          <t>material, mushroom, mushroomy</t>
-        </is>
-      </c>
-      <c r="O23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>HAVE</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Sweet Potato Pie</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>sweet_potato_pie</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Hayden</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr"/>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>Hayden</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr"/>
-      <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="3" t="inlineStr">
-        <is>
-          <t>baked_dessert, food, inn_plate</t>
-        </is>
-      </c>
-      <c r="O24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>HAVE</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Wild Berry Scone</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>wildberry_scone</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>Adeline</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>Adeline</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr"/>
-      <c r="M25" s="4" t="inlineStr"/>
-      <c r="N25" s="3" t="inlineStr">
-        <is>
-          <t>adept, baked_dessert, food, no_inn_plate</t>
-        </is>
-      </c>
-      <c r="O25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>CRAFT</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Ice Cream Sundae</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>ice_cream_sundae</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Butter [← 4× Milk]</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>Caldarus, Maple</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>Dell</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>Caldarus, Maple, Taliferro</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr"/>
-      <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="3" t="inlineStr">
-        <is>
-          <t>choco, food, frozen_dessert, no_inn_plate</t>
-        </is>
-      </c>
-      <c r="O26" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O26"/>
+  <autoFilter ref="A1:O20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2019,7 +1731,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
@@ -2124,7 +1836,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Wild Berry Scone</t>
+          <t>Lemonade</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -2183,7 +1895,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Frost Lily</t>
+          <t>Golden Cheesecake</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -2242,7 +1954,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Ice Cream Sundae</t>
+          <t>Golden Cheesecake</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2360,12 +2072,12 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Golden Cheesecake</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>LIKE</t>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -2419,12 +2131,12 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Glowberry Cookies</t>
+          <t>Jam Sandwich</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>LIKE</t>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -2478,12 +2190,12 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Cod</t>
+          <t>Dog Treat</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>LIKE</t>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -2537,12 +2249,12 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Peaches and Cream</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -2596,7 +2308,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Cherry Tart</t>
+          <t>Crystal Berry Pie</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2655,12 +2367,12 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Clam Chowder</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -2714,12 +2426,12 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Sweet Potato Pie</t>
+          <t>Golden Mayonnaise</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>LIKE</t>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -2773,7 +2485,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Incredibly Hot Pot</t>
+          <t>Crispy Fried Earthshroom</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -2832,12 +2544,12 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Grilled Corn</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>LIKE</t>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -2950,7 +2662,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Soy Sauce</t>
+          <t>Jam Sandwich</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3068,7 +2780,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Golden Horse Hair</t>
+          <t>Golden Cheesecake</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -3186,7 +2898,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Pond Skater</t>
+          <t>Jam Sandwich</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -3245,7 +2957,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Ice Cream Sundae</t>
+          <t>Pudding</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -3422,12 +3134,12 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Grilled Corn</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
@@ -3481,12 +3193,12 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Perfect Silver Ore</t>
+          <t>Miner's Mushroom Stew</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>LOVE</t>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
@@ -3540,12 +3252,12 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Breaded Catfish</t>
+          <t>Crystal Berry Pie</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>LOVE</t>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
@@ -3599,7 +3311,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Golden Horse Hair</t>
+          <t>Golden Cheesecake</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -3658,7 +3370,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Purple Mushroom</t>
+          <t>Monster Cookies</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -3717,7 +3429,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Fire Crystal</t>
+          <t>Crystal Berry Pie</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3776,7 +3488,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Glowberry Cookies</t>
+          <t>Golden Cheesecake</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3894,12 +3606,12 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Sweetroot</t>
+          <t>Deep Sea Soup</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>LIKE</t>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="H32" s="2" t="n">
@@ -3953,7 +3665,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Simmered Daikon</t>
+          <t>Crispy Fried Earthshroom</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -4012,7 +3724,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Golden Sheep Wool</t>
+          <t>Golden Cheesecake</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -4071,7 +3783,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Fennel</t>
+          <t>Miner's Mushroom Stew</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -16326,11 +16038,7 @@
           <t>breaded_catfish</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr"/>
@@ -16359,9 +16067,9 @@
       <c r="Y35" s="2" t="inlineStr"/>
       <c r="Z35" s="2" t="inlineStr"/>
       <c r="AA35" s="2" t="inlineStr"/>
-      <c r="AB35" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LOVE)</t>
+      <c r="AB35" s="9" t="inlineStr">
+        <is>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="AC35" s="2" t="inlineStr"/>
@@ -17984,11 +17692,7 @@
           <t>cherry_tart</t>
         </is>
       </c>
-      <c r="C65" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="2" t="inlineStr"/>
       <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr"/>
@@ -18001,9 +17705,9 @@
           <t>GIFTED</t>
         </is>
       </c>
-      <c r="L65" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="L65" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr"/>
@@ -18574,7 +18278,11 @@
           <t>clam_chowder</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr"/>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D75" s="2" t="inlineStr"/>
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr"/>
@@ -18584,9 +18292,9 @@
       <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr"/>
-      <c r="M75" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="M75" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr"/>
@@ -18885,20 +18593,16 @@
           <t>cod</t>
         </is>
       </c>
-      <c r="C80" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C80" s="2" t="inlineStr"/>
       <c r="D80" s="2" t="inlineStr"/>
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="2" t="inlineStr"/>
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr"/>
-      <c r="J80" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="J80" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr"/>
@@ -19840,7 +19544,11 @@
           <t>crispy_fried_earthshroom</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr"/>
+      <c r="C97" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D97" s="2" t="inlineStr"/>
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr"/>
@@ -19852,9 +19560,9 @@
       <c r="L97" s="2" t="inlineStr"/>
       <c r="M97" s="2" t="inlineStr"/>
       <c r="N97" s="2" t="inlineStr"/>
-      <c r="O97" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="O97" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="P97" s="2" t="inlineStr"/>
@@ -19876,9 +19584,9 @@
       <c r="AF97" s="2" t="inlineStr"/>
       <c r="AG97" s="2" t="inlineStr"/>
       <c r="AH97" s="2" t="inlineStr"/>
-      <c r="AI97" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="AI97" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="AJ97" s="2" t="inlineStr"/>
@@ -20182,7 +19890,11 @@
           <t>crystal_berry_pie</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr"/>
+      <c r="C103" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D103" s="2" t="inlineStr"/>
       <c r="E103" s="2" t="inlineStr"/>
       <c r="F103" s="2" t="inlineStr"/>
@@ -20195,9 +19907,9 @@
           <t>GIFTED</t>
         </is>
       </c>
-      <c r="L103" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="L103" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="M103" s="2" t="inlineStr"/>
@@ -20219,16 +19931,16 @@
       <c r="Y103" s="2" t="inlineStr"/>
       <c r="Z103" s="2" t="inlineStr"/>
       <c r="AA103" s="2" t="inlineStr"/>
-      <c r="AB103" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="AB103" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="AC103" s="2" t="inlineStr"/>
       <c r="AD103" s="2" t="inlineStr"/>
-      <c r="AE103" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="AE103" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="AF103" s="2" t="inlineStr"/>
@@ -20925,9 +20637,9 @@
           <t>PACK (LIKE)</t>
         </is>
       </c>
-      <c r="AH115" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="AH115" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="AI115" s="2" t="inlineStr"/>
@@ -21118,16 +20830,20 @@
           <t>dog_treat</t>
         </is>
       </c>
-      <c r="C119" s="2" t="inlineStr"/>
+      <c r="C119" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D119" s="2" t="inlineStr"/>
       <c r="E119" s="2" t="inlineStr"/>
       <c r="F119" s="2" t="inlineStr"/>
       <c r="G119" s="2" t="inlineStr"/>
       <c r="H119" s="2" t="inlineStr"/>
       <c r="I119" s="2" t="inlineStr"/>
-      <c r="J119" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="J119" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -21986,11 +21702,7 @@
           <t>fennel</t>
         </is>
       </c>
-      <c r="C135" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C135" s="2" t="inlineStr"/>
       <c r="D135" s="2" t="inlineStr"/>
       <c r="E135" s="2" t="inlineStr"/>
       <c r="F135" s="2" t="inlineStr"/>
@@ -22024,9 +21736,9 @@
       <c r="AH135" s="2" t="inlineStr"/>
       <c r="AI135" s="2" t="inlineStr"/>
       <c r="AJ135" s="2" t="inlineStr"/>
-      <c r="AK135" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="AK135" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
     </row>
@@ -22143,11 +21855,7 @@
           <t>fire_crystal</t>
         </is>
       </c>
-      <c r="C138" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C138" s="2" t="inlineStr"/>
       <c r="D138" s="2" t="inlineStr"/>
       <c r="E138" s="2" t="inlineStr"/>
       <c r="F138" s="2" t="inlineStr"/>
@@ -22175,9 +21883,9 @@
       <c r="AB138" s="2" t="inlineStr"/>
       <c r="AC138" s="2" t="inlineStr"/>
       <c r="AD138" s="2" t="inlineStr"/>
-      <c r="AE138" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LOVE)</t>
+      <c r="AE138" s="9" t="inlineStr">
+        <is>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="AF138" s="2" t="inlineStr"/>
@@ -22658,15 +22366,11 @@
           <t>frost_lily</t>
         </is>
       </c>
-      <c r="C147" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C147" s="2" t="inlineStr"/>
       <c r="D147" s="2" t="inlineStr"/>
-      <c r="E147" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr"/>
@@ -23110,19 +22814,15 @@
           <t>glowberry_cookies</t>
         </is>
       </c>
-      <c r="C155" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C155" s="2" t="inlineStr"/>
       <c r="D155" s="2" t="inlineStr"/>
       <c r="E155" s="2" t="inlineStr"/>
       <c r="F155" s="2" t="inlineStr"/>
       <c r="G155" s="2" t="inlineStr"/>
       <c r="H155" s="2" t="inlineStr"/>
-      <c r="I155" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="I155" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr"/>
@@ -23159,9 +22859,9 @@
       </c>
       <c r="AD155" s="2" t="inlineStr"/>
       <c r="AE155" s="2" t="inlineStr"/>
-      <c r="AF155" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="AF155" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="AG155" s="2" t="inlineStr"/>
@@ -23649,22 +23349,26 @@
           <t>golden_cheesecake</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr"/>
+      <c r="C164" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D164" s="2" t="inlineStr"/>
-      <c r="E164" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
-        </is>
-      </c>
-      <c r="F164" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="E164" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
+        </is>
+      </c>
+      <c r="F164" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr"/>
-      <c r="H164" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="H164" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="I164" s="2" t="inlineStr"/>
@@ -23682,9 +23386,9 @@
       <c r="Q164" s="2" t="inlineStr"/>
       <c r="R164" s="2" t="inlineStr"/>
       <c r="S164" s="2" t="inlineStr"/>
-      <c r="T164" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="T164" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="U164" s="2" t="inlineStr"/>
@@ -23695,24 +23399,24 @@
       <c r="Z164" s="2" t="inlineStr"/>
       <c r="AA164" s="2" t="inlineStr"/>
       <c r="AB164" s="2" t="inlineStr"/>
-      <c r="AC164" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="AC164" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="AD164" s="2" t="inlineStr"/>
       <c r="AE164" s="2" t="inlineStr"/>
-      <c r="AF164" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="AF164" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="AG164" s="2" t="inlineStr"/>
       <c r="AH164" s="2" t="inlineStr"/>
       <c r="AI164" s="2" t="inlineStr"/>
-      <c r="AJ164" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="AJ164" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="AK164" s="2" t="inlineStr"/>
@@ -24063,11 +23767,7 @@
           <t>golden_horse_hair</t>
         </is>
       </c>
-      <c r="C170" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C170" s="2" t="inlineStr"/>
       <c r="D170" s="2" t="inlineStr"/>
       <c r="E170" s="2" t="inlineStr"/>
       <c r="F170" s="2" t="inlineStr"/>
@@ -24084,9 +23784,9 @@
       <c r="Q170" s="2" t="inlineStr"/>
       <c r="R170" s="2" t="inlineStr"/>
       <c r="S170" s="2" t="inlineStr"/>
-      <c r="T170" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LOVE)</t>
+      <c r="T170" s="9" t="inlineStr">
+        <is>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="U170" s="8" t="inlineStr">
@@ -24105,9 +23805,9 @@
       <c r="Z170" s="2" t="inlineStr"/>
       <c r="AA170" s="2" t="inlineStr"/>
       <c r="AB170" s="2" t="inlineStr"/>
-      <c r="AC170" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LOVE)</t>
+      <c r="AC170" s="9" t="inlineStr">
+        <is>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="AD170" s="2" t="inlineStr"/>
@@ -24134,7 +23834,11 @@
           <t>golden_mayonnaise</t>
         </is>
       </c>
-      <c r="C171" s="2" t="inlineStr"/>
+      <c r="C171" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D171" s="2" t="inlineStr"/>
       <c r="E171" s="2" t="inlineStr"/>
       <c r="F171" s="2" t="inlineStr"/>
@@ -24145,9 +23849,9 @@
       <c r="K171" s="2" t="inlineStr"/>
       <c r="L171" s="2" t="inlineStr"/>
       <c r="M171" s="2" t="inlineStr"/>
-      <c r="N171" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="N171" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="O171" s="2" t="inlineStr"/>
@@ -24411,9 +24115,9 @@
       <c r="AG175" s="2" t="inlineStr"/>
       <c r="AH175" s="2" t="inlineStr"/>
       <c r="AI175" s="2" t="inlineStr"/>
-      <c r="AJ175" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="AJ175" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="AK175" s="2" t="inlineStr"/>
@@ -24708,7 +24412,11 @@
           <t>grilled_corn</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr"/>
+      <c r="C181" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D181" s="2" t="inlineStr"/>
       <c r="E181" s="2" t="inlineStr"/>
       <c r="F181" s="2" t="inlineStr"/>
@@ -24725,9 +24433,9 @@
       <c r="M181" s="2" t="inlineStr"/>
       <c r="N181" s="2" t="inlineStr"/>
       <c r="O181" s="2" t="inlineStr"/>
-      <c r="P181" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="P181" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="Q181" s="2" t="inlineStr"/>
@@ -24739,9 +24447,9 @@
       <c r="W181" s="2" t="inlineStr"/>
       <c r="X181" s="2" t="inlineStr"/>
       <c r="Y181" s="2" t="inlineStr"/>
-      <c r="Z181" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="Z181" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="AA181" s="2" t="inlineStr"/>
@@ -25640,16 +25348,12 @@
           <t>ice_cream_sundae</t>
         </is>
       </c>
-      <c r="C197" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C197" s="2" t="inlineStr"/>
       <c r="D197" s="2" t="inlineStr"/>
       <c r="E197" s="2" t="inlineStr"/>
-      <c r="F197" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="F197" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr"/>
@@ -25676,9 +25380,9 @@
       <c r="T197" s="2" t="inlineStr"/>
       <c r="U197" s="2" t="inlineStr"/>
       <c r="V197" s="2" t="inlineStr"/>
-      <c r="W197" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="W197" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="X197" s="2" t="inlineStr"/>
@@ -25821,11 +25525,7 @@
           <t>incredibly_hot_pot</t>
         </is>
       </c>
-      <c r="C200" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C200" s="2" t="inlineStr"/>
       <c r="D200" s="2" t="inlineStr"/>
       <c r="E200" s="2" t="inlineStr"/>
       <c r="F200" s="10" t="inlineStr">
@@ -25841,9 +25541,9 @@
       <c r="L200" s="2" t="inlineStr"/>
       <c r="M200" s="2" t="inlineStr"/>
       <c r="N200" s="2" t="inlineStr"/>
-      <c r="O200" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LOVE)</t>
+      <c r="O200" s="9" t="inlineStr">
+        <is>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="P200" s="2" t="inlineStr"/>
@@ -26061,15 +25761,19 @@
           <t>jam_sandwich</t>
         </is>
       </c>
-      <c r="C204" s="2" t="inlineStr"/>
+      <c r="C204" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D204" s="2" t="inlineStr"/>
       <c r="E204" s="2" t="inlineStr"/>
       <c r="F204" s="2" t="inlineStr"/>
       <c r="G204" s="2" t="inlineStr"/>
       <c r="H204" s="2" t="inlineStr"/>
-      <c r="I204" s="9" t="inlineStr">
-        <is>
-          <t>LOVE</t>
+      <c r="I204" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LOVE)</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr"/>
@@ -26080,17 +25784,17 @@
       <c r="O204" s="2" t="inlineStr"/>
       <c r="P204" s="2" t="inlineStr"/>
       <c r="Q204" s="2" t="inlineStr"/>
-      <c r="R204" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="R204" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="S204" s="2" t="inlineStr"/>
       <c r="T204" s="2" t="inlineStr"/>
       <c r="U204" s="2" t="inlineStr"/>
-      <c r="V204" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="V204" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="W204" s="8" t="inlineStr">
@@ -26588,10 +26292,14 @@
           <t>lemonade</t>
         </is>
       </c>
-      <c r="C213" s="2" t="inlineStr"/>
-      <c r="D213" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="C213" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
+      <c r="D213" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr"/>
@@ -27421,7 +27129,11 @@
           <t>miners_mushroom_stew</t>
         </is>
       </c>
-      <c r="C228" s="2" t="inlineStr"/>
+      <c r="C228" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D228" s="2" t="inlineStr"/>
       <c r="E228" s="2" t="inlineStr"/>
       <c r="F228" s="2" t="inlineStr"/>
@@ -27449,9 +27161,9 @@
       <c r="X228" s="2" t="inlineStr"/>
       <c r="Y228" s="2" t="inlineStr"/>
       <c r="Z228" s="2" t="inlineStr"/>
-      <c r="AA228" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="AA228" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="AB228" s="8" t="inlineStr">
@@ -27467,9 +27179,9 @@
       <c r="AH228" s="2" t="inlineStr"/>
       <c r="AI228" s="2" t="inlineStr"/>
       <c r="AJ228" s="2" t="inlineStr"/>
-      <c r="AK228" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="AK228" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
     </row>
@@ -27814,7 +27526,11 @@
           <t>monster_cookie</t>
         </is>
       </c>
-      <c r="C235" s="2" t="inlineStr"/>
+      <c r="C235" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D235" s="2" t="inlineStr"/>
       <c r="E235" s="2" t="inlineStr"/>
       <c r="F235" s="2" t="inlineStr"/>
@@ -27849,9 +27565,9 @@
       <c r="AA235" s="2" t="inlineStr"/>
       <c r="AB235" s="2" t="inlineStr"/>
       <c r="AC235" s="2" t="inlineStr"/>
-      <c r="AD235" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="AD235" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="AE235" s="10" t="inlineStr">
@@ -29158,18 +28874,14 @@
           <t>orange</t>
         </is>
       </c>
-      <c r="C259" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C259" s="2" t="inlineStr"/>
       <c r="D259" s="2" t="inlineStr"/>
       <c r="E259" s="2" t="inlineStr"/>
       <c r="F259" s="2" t="inlineStr"/>
       <c r="G259" s="2" t="inlineStr"/>
-      <c r="H259" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="H259" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="I259" s="2" t="inlineStr"/>
@@ -29179,9 +28891,9 @@
       <c r="M259" s="2" t="inlineStr"/>
       <c r="N259" s="2" t="inlineStr"/>
       <c r="O259" s="2" t="inlineStr"/>
-      <c r="P259" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="P259" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="Q259" s="2" t="inlineStr"/>
@@ -29606,7 +29318,11 @@
           <t>peaches_and_cream</t>
         </is>
       </c>
-      <c r="C267" s="2" t="inlineStr"/>
+      <c r="C267" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D267" s="8" t="inlineStr">
         <is>
           <t>GIFTED</t>
@@ -29618,9 +29334,9 @@
       <c r="H267" s="2" t="inlineStr"/>
       <c r="I267" s="2" t="inlineStr"/>
       <c r="J267" s="2" t="inlineStr"/>
-      <c r="K267" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="K267" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="L267" s="2" t="inlineStr"/>
@@ -30444,11 +30160,7 @@
           <t>perfect_silver_ore</t>
         </is>
       </c>
-      <c r="C281" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C281" s="2" t="inlineStr"/>
       <c r="D281" s="2" t="inlineStr"/>
       <c r="E281" s="2" t="inlineStr"/>
       <c r="F281" s="2" t="inlineStr"/>
@@ -30476,9 +30188,9 @@
       </c>
       <c r="Y281" s="2" t="inlineStr"/>
       <c r="Z281" s="2" t="inlineStr"/>
-      <c r="AA281" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LOVE)</t>
+      <c r="AA281" s="9" t="inlineStr">
+        <is>
+          <t>LOVE</t>
         </is>
       </c>
       <c r="AB281" s="2" t="inlineStr"/>
@@ -31132,11 +30844,7 @@
           <t>pond_skater</t>
         </is>
       </c>
-      <c r="C293" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C293" s="2" t="inlineStr"/>
       <c r="D293" s="2" t="inlineStr"/>
       <c r="E293" s="2" t="inlineStr"/>
       <c r="F293" s="2" t="inlineStr"/>
@@ -31155,9 +30863,9 @@
       <c r="S293" s="2" t="inlineStr"/>
       <c r="T293" s="2" t="inlineStr"/>
       <c r="U293" s="2" t="inlineStr"/>
-      <c r="V293" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="V293" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="W293" s="2" t="inlineStr"/>
@@ -31289,7 +30997,11 @@
           <t>pudding</t>
         </is>
       </c>
-      <c r="C296" s="2" t="inlineStr"/>
+      <c r="C296" s="11" t="inlineStr">
+        <is>
+          <t>IN BAG TODAY</t>
+        </is>
+      </c>
       <c r="D296" s="2" t="inlineStr"/>
       <c r="E296" s="2" t="inlineStr"/>
       <c r="F296" s="2" t="inlineStr"/>
@@ -31317,9 +31029,9 @@
       <c r="T296" s="2" t="inlineStr"/>
       <c r="U296" s="2" t="inlineStr"/>
       <c r="V296" s="2" t="inlineStr"/>
-      <c r="W296" s="10" t="inlineStr">
-        <is>
-          <t>LIKE</t>
+      <c r="W296" s="11" t="inlineStr">
+        <is>
+          <t>PACK (LIKE)</t>
         </is>
       </c>
       <c r="X296" s="2" t="inlineStr"/>
@@ -31584,11 +31296,7 @@
           <t>purple_mushroom</t>
         </is>
       </c>
-      <c r="C301" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C301" s="2" t="inlineStr"/>
       <c r="D301" s="2" t="inlineStr"/>
       <c r="E301" s="2" t="inlineStr"/>
       <c r="F301" s="2" t="inlineStr"/>
@@ -31615,9 +31323,9 @@
       <c r="AA301" s="2" t="inlineStr"/>
       <c r="AB301" s="2" t="inlineStr"/>
       <c r="AC301" s="2" t="inlineStr"/>
-      <c r="AD301" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="AD301" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="AE301" s="2" t="inlineStr"/>
@@ -34625,11 +34333,7 @@
           <t>simmered_daikon</t>
         </is>
       </c>
-      <c r="C356" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C356" s="2" t="inlineStr"/>
       <c r="D356" s="2" t="inlineStr"/>
       <c r="E356" s="2" t="inlineStr"/>
       <c r="F356" s="2" t="inlineStr"/>
@@ -34665,9 +34369,9 @@
       <c r="AF356" s="2" t="inlineStr"/>
       <c r="AG356" s="2" t="inlineStr"/>
       <c r="AH356" s="2" t="inlineStr"/>
-      <c r="AI356" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="AI356" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="AJ356" s="2" t="inlineStr"/>
@@ -35108,11 +34812,7 @@
           <t>soy_sauce</t>
         </is>
       </c>
-      <c r="C365" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C365" s="2" t="inlineStr"/>
       <c r="D365" s="2" t="inlineStr"/>
       <c r="E365" s="2" t="inlineStr"/>
       <c r="F365" s="2" t="inlineStr"/>
@@ -35127,9 +34827,9 @@
       <c r="O365" s="2" t="inlineStr"/>
       <c r="P365" s="2" t="inlineStr"/>
       <c r="Q365" s="2" t="inlineStr"/>
-      <c r="R365" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="R365" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="S365" s="2" t="inlineStr"/>
@@ -36618,11 +36318,7 @@
           <t>sweet_potato_pie</t>
         </is>
       </c>
-      <c r="C391" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C391" s="2" t="inlineStr"/>
       <c r="D391" s="2" t="inlineStr"/>
       <c r="E391" s="2" t="inlineStr"/>
       <c r="F391" s="2" t="inlineStr"/>
@@ -36633,9 +36329,9 @@
       <c r="K391" s="2" t="inlineStr"/>
       <c r="L391" s="2" t="inlineStr"/>
       <c r="M391" s="2" t="inlineStr"/>
-      <c r="N391" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="N391" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="O391" s="2" t="inlineStr"/>
@@ -36732,11 +36428,7 @@
           <t>sweetroot</t>
         </is>
       </c>
-      <c r="C393" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
+      <c r="C393" s="2" t="inlineStr"/>
       <c r="D393" s="2" t="inlineStr"/>
       <c r="E393" s="2" t="inlineStr"/>
       <c r="F393" s="2" t="inlineStr"/>
@@ -36775,9 +36467,9 @@
       <c r="AE393" s="2" t="inlineStr"/>
       <c r="AF393" s="2" t="inlineStr"/>
       <c r="AG393" s="2" t="inlineStr"/>
-      <c r="AH393" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="AH393" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="AI393" s="2" t="inlineStr"/>
@@ -38925,14 +38617,10 @@
           <t>wildberry_scone</t>
         </is>
       </c>
-      <c r="C432" s="11" t="inlineStr">
-        <is>
-          <t>IN BAG TODAY</t>
-        </is>
-      </c>
-      <c r="D432" s="11" t="inlineStr">
-        <is>
-          <t>PACK (LIKE)</t>
+      <c r="C432" s="2" t="inlineStr"/>
+      <c r="D432" s="10" t="inlineStr">
+        <is>
+          <t>LIKE</t>
         </is>
       </c>
       <c r="E432" s="2" t="inlineStr"/>
@@ -39370,4 +39058,137 @@
   <autoFilter ref="A1:AK439"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Recipe Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unlock Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Perch Risotto</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Request Board: Errol's Request for Perch</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Incredibly Hot Pot</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>The Lava Caves (Taste Maker Perk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Wild Berry Pie</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Request Board: Reina's Request for Berries</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Loaded Baked Potato</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Request Board: Hayden's Request for Baked Potato</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Strawberry Shortcake</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Request Board: Eiland's Request for a Strawberry</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>